<commit_message>
Daily NSE scan: 2026-09-02
</commit_message>
<xml_diff>
--- a/output/2026-09-02/enriched_analysis.xlsx
+++ b/output/2026-09-02/enriched_analysis.xlsx
@@ -616,7 +616,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GANDHAR OIL REFINERY (INDIA) LIMITED</t>
+          <t>Gandhar Oil Refinery (India) Limited</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
+          <t>Ganesh Consumer Products Limited</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GANDHAR OIL REFINERY (INDIA) LIMITED</t>
+          <t>Gandhar Oil Refinery (India) Limited</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -6267,7 +6267,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GANESH CONSUMER PRODUCTS LIMITED</t>
+          <t>Ganesh Consumer Products Limited</t>
         </is>
       </c>
       <c r="C32" t="n">

</xml_diff>